<commit_message>
corrige intensivo extensivo y agrega treemaps
</commit_message>
<xml_diff>
--- a/output/reporte/resultados_complexity_final.xlsx
+++ b/output/reporte/resultados_complexity_final.xlsx
@@ -18921,12 +18921,12 @@
       </c>
       <c r="E54" s="1" t="inlineStr">
         <is>
-          <t>2822</t>
+          <t>2819</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Fabricación de maquinaria para la conformación de metales y de máquinas herramienta</t>
+          <t>Fabricación de otros tipos de maquinaria de uso general</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -18970,12 +18970,12 @@
       </c>
       <c r="E55" s="1" t="inlineStr">
         <is>
-          <t>2819</t>
+          <t>2822</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Fabricación de otros tipos de maquinaria de uso general</t>
+          <t>Fabricación de maquinaria para la conformación de metales y de máquinas herramienta</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">

</xml_diff>